<commit_message>
Updates to differentriate insurance costs by vehicle technology and uses newer data
</commit_message>
<xml_diff>
--- a/InputData/trans/AVIC/Annual Vehicle Insurance Cost.xlsx
+++ b/InputData/trans/AVIC/Annual Vehicle Insurance Cost.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeff Rissman\CodeRepositories\eps-us\InputData\trans\AVIC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\trans\AVIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C68CA1-D4E5-4267-A93A-22A2147EC345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E74BD3-8B7E-4AA4-A3CF-42FF8ECD662A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12870" yWindow="1470" windowWidth="22500" windowHeight="21135" xr2:uid="{D78DFE5E-0A7F-4A12-AD34-4FEABB0CFCE7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{D78DFE5E-0A7F-4A12-AD34-4FEABB0CFCE7}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Data" sheetId="3" r:id="rId2"/>
-    <sheet name="AVIC" sheetId="2" r:id="rId3"/>
+    <sheet name="AVIC-passenger" sheetId="2" r:id="rId3"/>
+    <sheet name="AVIC-freight" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="83">
   <si>
     <t>AVIC Annual Vehicle Insurance Cost</t>
   </si>
@@ -44,18 +45,9 @@
     <t>Source:</t>
   </si>
   <si>
-    <t>American Automobile Association</t>
-  </si>
-  <si>
     <t>LDVs</t>
   </si>
   <si>
-    <t>Average Annual Cost of New Car Ownership Increases 5% to $9,282</t>
-  </si>
-  <si>
-    <t>https://www.aaa.com/autorepair/articles/average-annual-cost-of-new-vehicle-ownership</t>
-  </si>
-  <si>
     <t>HDVs</t>
   </si>
   <si>
@@ -71,18 +63,6 @@
     <t>motorbikes</t>
   </si>
   <si>
-    <t>passenger</t>
-  </si>
-  <si>
-    <t>freight</t>
-  </si>
-  <si>
-    <t>Data from AAA:</t>
-  </si>
-  <si>
-    <t>$/yr (2019 USD)</t>
-  </si>
-  <si>
     <t>Freight HDVs</t>
   </si>
   <si>
@@ -182,9 +162,6 @@
     <t>For freight LDVs, the value for "cargo or delivery van" is most appropriate.</t>
   </si>
   <si>
-    <t>Passenger LDV</t>
-  </si>
-  <si>
     <t>Passenger Motorbikes</t>
   </si>
   <si>
@@ -239,13 +216,76 @@
     <t>2020 to 2012 USD</t>
   </si>
   <si>
-    <t>2021 to 2012 USD (est.)</t>
-  </si>
-  <si>
-    <t>Est. 2021 inflation rate (from BLS, through Nov 2021, https://www.bls.gov/cpi/)</t>
-  </si>
-  <si>
     <t>2012 USD/year</t>
+  </si>
+  <si>
+    <t>Data from Insurify:</t>
+  </si>
+  <si>
+    <t>Passenger LDV, gasoline</t>
+  </si>
+  <si>
+    <t>Passenger LDV, battery electric</t>
+  </si>
+  <si>
+    <t>$/yr (2025 USD)</t>
+  </si>
+  <si>
+    <t>battery electric vehicle</t>
+  </si>
+  <si>
+    <t>natural gas vehicle</t>
+  </si>
+  <si>
+    <t>gasoline vehicle</t>
+  </si>
+  <si>
+    <t>diesel vehicle</t>
+  </si>
+  <si>
+    <t>plugin hybrid vehicle</t>
+  </si>
+  <si>
+    <t>LPG vehicle</t>
+  </si>
+  <si>
+    <t>hydrogen vehicle</t>
+  </si>
+  <si>
+    <t>2025 to 2012 USD</t>
+  </si>
+  <si>
+    <t>2021 to 2012 USD</t>
+  </si>
+  <si>
+    <t>Insurify</t>
+  </si>
+  <si>
+    <t>https://insurify.com/car-insurance/report/electric-vehicle-insurance-costs/</t>
+  </si>
+  <si>
+    <t>EVs Cost 49% More to Insure Than Gas-Powered Cars, Data Reveals</t>
+  </si>
+  <si>
+    <t>BEV Markup for Freight LDVs/HDVs and Passenger HDVs</t>
+  </si>
+  <si>
+    <t>CCJ</t>
+  </si>
+  <si>
+    <t>Why zero-emission trucks often cost 30-50% more to insure than diesel models</t>
+  </si>
+  <si>
+    <t>https://www.ccjdigital.com/business/article/15753084/why-zeroemission-truck-insurance-costs-can-wipe-out-fuel-savings</t>
+  </si>
+  <si>
+    <t>We apply a markup ratio of 40% for BEV passenger HDVs and freight LDVs/HDVs based on the CCJ article.</t>
+  </si>
+  <si>
+    <t>We take the average of BEV and gasoline vehicle for PHEV. For LPG and hydrogen, we use BEV costs</t>
+  </si>
+  <si>
+    <t>as these are newer technologies (and H2 vehicles are effectively BEVs but use a fuel cell).</t>
   </si>
 </sst>
 </file>
@@ -280,7 +320,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -305,6 +345,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -319,7 +383,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -336,9 +400,13 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -358,9 +426,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -398,7 +466,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -504,7 +572,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -646,7 +714,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -654,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC790369-4F84-43C0-97E9-6D0C01E4139F}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -670,37 +738,37 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>2</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
-        <v>2019</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>5</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -710,179 +778,221 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <v>2021</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>55</v>
+      <c r="B33" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>56</v>
+      <c r="B34" s="3">
+        <v>2025</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>58</v>
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>59</v>
+      <c r="A38" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>63</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>64</v>
+      <c r="A44" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46">
+      <c r="A46" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
         <v>0.89800000000000002</v>
       </c>
-      <c r="B46" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47">
+      <c r="B58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
         <v>0.88700000000000001</v>
       </c>
-      <c r="B47" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="10">
-        <f>A47/(1+A50)</f>
-        <v>0.83052434456928836</v>
-      </c>
-      <c r="B48" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="9">
-        <v>6.8000000000000005E-2</v>
-      </c>
-      <c r="B50" t="s">
-        <v>68</v>
-      </c>
+      <c r="B59" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="10">
+        <v>0.84730412960844359</v>
+      </c>
+      <c r="B60" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>0.71310900044104586</v>
+      </c>
+      <c r="B61" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" xr:uid="{E31DF05E-B87F-4D1B-AC11-F88AEEDA7D2F}"/>
-    <hyperlink ref="B19" r:id="rId2" xr:uid="{DC3E2816-48AF-4FA2-A726-B61F86FC64CE}"/>
-    <hyperlink ref="B24" r:id="rId3" xr:uid="{929BA16D-4044-4610-8C77-D354B466069A}"/>
-    <hyperlink ref="B13" r:id="rId4" xr:uid="{3786F80B-C165-478C-A885-8E7EE782E47E}"/>
-    <hyperlink ref="B30" r:id="rId5" xr:uid="{ECB38255-597D-4E40-A940-86F690DADDBD}"/>
+    <hyperlink ref="B19" r:id="rId1" xr:uid="{DC3E2816-48AF-4FA2-A726-B61F86FC64CE}"/>
+    <hyperlink ref="B24" r:id="rId2" xr:uid="{929BA16D-4044-4610-8C77-D354B466069A}"/>
+    <hyperlink ref="B13" r:id="rId3" xr:uid="{3786F80B-C165-478C-A885-8E7EE782E47E}"/>
+    <hyperlink ref="B30" r:id="rId4" xr:uid="{ECB38255-597D-4E40-A940-86F690DADDBD}"/>
+    <hyperlink ref="B36" r:id="rId5" xr:uid="{36CC9A78-2687-4407-AACA-D5FF51BD9AC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId6"/>
@@ -891,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C907FFC-9E03-403C-A103-2A580B24C105}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" customWidth="1"/>
@@ -900,247 +1010,258 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B4" s="8">
-        <v>1194</v>
+        <v>2732</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="8">
+        <v>4058</v>
+      </c>
+      <c r="C5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="D11" t="s">
         <v>38</v>
-      </c>
-      <c r="B11">
-        <v>600</v>
-      </c>
-      <c r="C11">
-        <v>2400</v>
-      </c>
-      <c r="D11">
-        <f>AVERAGE(B11:C11)</f>
-        <v>1500</v>
-      </c>
-      <c r="E11" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12">
+        <v>600</v>
+      </c>
+      <c r="C12">
+        <v>2400</v>
+      </c>
+      <c r="D12">
+        <f>AVERAGE(B12:C12)</f>
+        <v>1500</v>
+      </c>
+      <c r="E12" t="s">
         <v>39</v>
-      </c>
-      <c r="B12">
-        <v>4000</v>
-      </c>
-      <c r="C12">
-        <v>10000</v>
-      </c>
-      <c r="D12">
-        <f t="shared" ref="D12:D15" si="0">AVERAGE(B12:C12)</f>
-        <v>7000</v>
-      </c>
-      <c r="E12" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B13">
+        <v>4000</v>
+      </c>
+      <c r="C13">
+        <v>10000</v>
+      </c>
+      <c r="D13">
+        <f t="shared" ref="D13:D16" si="0">AVERAGE(B13:C13)</f>
+        <v>7000</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14">
         <v>3300</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>6200</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D14" s="8">
         <f t="shared" si="0"/>
         <v>4750</v>
       </c>
-      <c r="E13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14">
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15">
         <v>5000</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>10000</v>
       </c>
-      <c r="D14">
+      <c r="D15">
         <f t="shared" si="0"/>
         <v>7500</v>
       </c>
-      <c r="E14" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15">
+      <c r="E15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16">
         <v>8000</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>12500</v>
       </c>
-      <c r="D15">
+      <c r="D16">
         <f t="shared" si="0"/>
         <v>10250</v>
       </c>
-      <c r="E15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21">
-        <v>640</v>
-      </c>
-      <c r="C21" t="s">
-        <v>20</v>
-      </c>
+      <c r="E16" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B22">
-        <v>982</v>
+        <v>640</v>
       </c>
       <c r="C22" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B23">
-        <f>AVERAGE(B21:B22)</f>
-        <v>811</v>
+        <v>982</v>
       </c>
       <c r="C23" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="8">
-        <f>B23*12</f>
+        <v>16</v>
+      </c>
+      <c r="B24">
+        <f>AVERAGE(B22:B23)</f>
+        <v>811</v>
+      </c>
+      <c r="C24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="8">
+        <f>B24*12</f>
         <v>9732</v>
       </c>
-      <c r="C24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>27</v>
+      <c r="C25" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="8">
         <v>9420</v>
       </c>
-      <c r="C31" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>30</v>
-      </c>
-      <c r="B37" s="8">
+      <c r="C32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="8">
         <v>721</v>
       </c>
-      <c r="C37" t="s">
-        <v>46</v>
+      <c r="C38" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1151,94 +1272,476 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2702F2D4-8FE2-493C-8905-78A0E4F67148}">
   <sheetPr>
-    <tabColor theme="4" tint="-0.249977111117893"/>
+    <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
-    <col min="2" max="3" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="H1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="13">
+        <f>Data!B5*About!A61</f>
+        <v>2893.7963237897643</v>
+      </c>
+      <c r="C2" s="17">
+        <f>D2</f>
+        <v>1948.2137892049373</v>
+      </c>
+      <c r="D2" s="12">
+        <f>Data!B4*About!A61</f>
+        <v>1948.2137892049373</v>
+      </c>
+      <c r="E2" s="16">
+        <f>D2</f>
+        <v>1948.2137892049373</v>
+      </c>
+      <c r="F2" s="13">
+        <f>AVERAGE(D2,B2)</f>
+        <v>2421.0050564973508</v>
+      </c>
+      <c r="G2" s="14">
+        <f>D2</f>
+        <v>1948.2137892049373</v>
+      </c>
+      <c r="H2" s="15">
+        <f>B2</f>
+        <v>2893.7963237897643</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="11">
-        <f>Data!B4*About!A46</f>
-        <v>1072.212</v>
+      <c r="B3" s="11">
+        <f>D3*1.4</f>
+        <v>11174.246861276153</v>
+      </c>
+      <c r="C3" s="11">
+        <f>D3</f>
+        <v>7981.6049009115386</v>
+      </c>
+      <c r="D3" s="18">
+        <f>Data!B32*About!A60</f>
+        <v>7981.6049009115386</v>
+      </c>
+      <c r="E3" s="18">
+        <f t="shared" ref="D3:H3" si="0">D3</f>
+        <v>7981.6049009115386</v>
+      </c>
+      <c r="F3" s="18">
+        <f>AVERAGE(D3,B3)</f>
+        <v>9577.9258810938463</v>
+      </c>
+      <c r="G3" s="11">
+        <f>D3</f>
+        <v>7981.6049009115386</v>
+      </c>
+      <c r="H3" s="11">
+        <f>B3</f>
+        <v>11174.246861276153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="11">
+        <f t="shared" ref="C4:H4" si="1">B4</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E4" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F4" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G4" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H4" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5" s="11">
+        <f t="shared" ref="C5:H5" si="2">B5</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="11">
+        <f t="shared" ref="C6:H6" si="3">B6</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="11">
+        <f>Data!B38*About!A60</f>
+        <v>610.90627744768778</v>
+      </c>
+      <c r="C7" s="11">
+        <f t="shared" ref="C7:H7" si="4">B7</f>
+        <v>610.90627744768778</v>
+      </c>
+      <c r="D7" s="11">
+        <f t="shared" si="4"/>
+        <v>610.90627744768778</v>
+      </c>
+      <c r="E7" s="11">
+        <f t="shared" si="4"/>
+        <v>610.90627744768778</v>
+      </c>
+      <c r="F7" s="11">
+        <f t="shared" si="4"/>
+        <v>610.90627744768778</v>
+      </c>
+      <c r="G7" s="11">
+        <f t="shared" si="4"/>
+        <v>610.90627744768778</v>
+      </c>
+      <c r="H7" s="11">
+        <f t="shared" si="4"/>
+        <v>610.90627744768778</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98AA8790-CEA3-4C44-81E1-FC7A1C5ACA24}">
+  <sheetPr>
+    <tabColor rgb="FF002060"/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <f>E2*1.4</f>
+        <v>5634.5724618961494</v>
       </c>
       <c r="C2" s="11">
-        <f>Data!D13*About!A48</f>
-        <v>3944.9906367041199</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <f>E2</f>
+        <v>4024.6946156401073</v>
+      </c>
+      <c r="D2" s="11">
+        <f>E2</f>
+        <v>4024.6946156401073</v>
+      </c>
+      <c r="E2" s="11">
+        <f>Data!D14*About!A60</f>
+        <v>4024.6946156401073</v>
+      </c>
+      <c r="F2" s="11">
+        <f>AVERAGE(E2,B2)</f>
+        <v>4829.6335387681283</v>
+      </c>
+      <c r="G2">
+        <f>B2</f>
+        <v>5634.5724618961494</v>
+      </c>
+      <c r="H2">
+        <f>B2</f>
+        <v>5634.5724618961494</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <f>E3*1.4</f>
+        <v>11544.349305089121</v>
+      </c>
+      <c r="C3" s="11">
+        <f t="shared" ref="C3:C7" si="0">E3</f>
+        <v>8245.9637893493727</v>
+      </c>
+      <c r="D3" s="11">
+        <f t="shared" ref="D3:D7" si="1">E3</f>
+        <v>8245.9637893493727</v>
+      </c>
+      <c r="E3" s="11">
+        <f>Data!B25*About!A60</f>
+        <v>8245.9637893493727</v>
+      </c>
+      <c r="F3" s="11">
+        <f t="shared" ref="F3:F7" si="2">AVERAGE(E3,B3)</f>
+        <v>9895.1565472192469</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G7" si="3">B3</f>
+        <v>11544.349305089121</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H7" si="4">B3</f>
+        <v>11544.349305089121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <f>E4</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D4" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <f t="shared" ref="B5:B7" si="5">E5</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D5" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="11">
-        <f>Data!B31*About!A48</f>
-        <v>7823.5393258426966</v>
-      </c>
-      <c r="C3" s="11">
-        <f>Data!B24*About!A48</f>
-        <v>8082.6629213483147</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B6">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="C6" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D6" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="11">
-        <f>Data!B37*About!A48</f>
-        <v>598.80805243445695</v>
-      </c>
-      <c r="C7">
+      <c r="B7">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="C7" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D7" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>